<commit_message>
fix: Los-Teileingabe ohne #NV, Excel rechnet beim Öffnen neu
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vorlage/stammtisch-turnier.xlsx
+++ b/vorlage/stammtisch-turnier.xlsx
@@ -13,7 +13,7 @@
     <sheet sheetId="7" name="Endplatzierung" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="Spieler" state="visible" r:id="rId11"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -2484,7 +2484,7 @@
         <f>J10*10^11+(I10+500)*10^8+U10*10^6+(V10+500)*10^3+G10</f>
       </c>
       <c r="Y10" s="5">
-        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X10))+SUMPRODUCT(($X$10:$X$14=X10)*($W$10:$W$14&lt;&gt;"")*(W10&lt;&gt;"")*($W$10:$W$14&lt;W10))</f>
+        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X10))+SUMPRODUCT(($X$10:$X$14=X10)*($W$10:$W$14&lt;W10))</f>
       </c>
       <c r="Z10" s="5">
         <f>IF(SUMPRODUCT(($X$10:$X$14=X10)*($A$10:$A$14&lt;&gt;A10)*((($W$10:$W$14="")+(W10="")+($W$10:$W$14=W10))&gt;0))&gt;0,1,0)</f>
@@ -2567,7 +2567,7 @@
         <f>J11*10^11+(I11+500)*10^8+U11*10^6+(V11+500)*10^3+G11</f>
       </c>
       <c r="Y11" s="5">
-        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X11))+SUMPRODUCT(($X$10:$X$14=X11)*($W$10:$W$14&lt;&gt;"")*(W11&lt;&gt;"")*($W$10:$W$14&lt;W11))</f>
+        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X11))+SUMPRODUCT(($X$10:$X$14=X11)*($W$10:$W$14&lt;W11))</f>
       </c>
       <c r="Z11" s="5">
         <f>IF(SUMPRODUCT(($X$10:$X$14=X11)*($A$10:$A$14&lt;&gt;A11)*((($W$10:$W$14="")+(W11="")+($W$10:$W$14=W11))&gt;0))&gt;0,1,0)</f>
@@ -2650,7 +2650,7 @@
         <f>J12*10^11+(I12+500)*10^8+U12*10^6+(V12+500)*10^3+G12</f>
       </c>
       <c r="Y12" s="5">
-        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X12))+SUMPRODUCT(($X$10:$X$14=X12)*($W$10:$W$14&lt;&gt;"")*(W12&lt;&gt;"")*($W$10:$W$14&lt;W12))</f>
+        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X12))+SUMPRODUCT(($X$10:$X$14=X12)*($W$10:$W$14&lt;W12))</f>
       </c>
       <c r="Z12" s="5">
         <f>IF(SUMPRODUCT(($X$10:$X$14=X12)*($A$10:$A$14&lt;&gt;A12)*((($W$10:$W$14="")+(W12="")+($W$10:$W$14=W12))&gt;0))&gt;0,1,0)</f>
@@ -2733,7 +2733,7 @@
         <f>J13*10^11+(I13+500)*10^8+U13*10^6+(V13+500)*10^3+G13</f>
       </c>
       <c r="Y13" s="5">
-        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X13))+SUMPRODUCT(($X$10:$X$14=X13)*($W$10:$W$14&lt;&gt;"")*(W13&lt;&gt;"")*($W$10:$W$14&lt;W13))</f>
+        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X13))+SUMPRODUCT(($X$10:$X$14=X13)*($W$10:$W$14&lt;W13))</f>
       </c>
       <c r="Z13" s="5">
         <f>IF(SUMPRODUCT(($X$10:$X$14=X13)*($A$10:$A$14&lt;&gt;A13)*((($W$10:$W$14="")+(W13="")+($W$10:$W$14=W13))&gt;0))&gt;0,1,0)</f>
@@ -2816,7 +2816,7 @@
         <f>J14*10^11+(I14+500)*10^8+U14*10^6+(V14+500)*10^3+G14</f>
       </c>
       <c r="Y14" s="5">
-        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X14))+SUMPRODUCT(($X$10:$X$14=X14)*($W$10:$W$14&lt;&gt;"")*(W14&lt;&gt;"")*($W$10:$W$14&lt;W14))</f>
+        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X14))+SUMPRODUCT(($X$10:$X$14=X14)*($W$10:$W$14&lt;W14))</f>
       </c>
       <c r="Z14" s="5">
         <f>IF(SUMPRODUCT(($X$10:$X$14=X14)*($A$10:$A$14&lt;&gt;A14)*((($W$10:$W$14="")+(W14="")+($W$10:$W$14=W14))&gt;0))&gt;0,1,0)</f>
@@ -3280,7 +3280,7 @@
         <f>J10*10^11+(I10+500)*10^8+U10*10^6+(V10+500)*10^3+G10</f>
       </c>
       <c r="Y10" s="5">
-        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X10))+SUMPRODUCT(($X$10:$X$14=X10)*($W$10:$W$14&lt;&gt;"")*(W10&lt;&gt;"")*($W$10:$W$14&lt;W10))</f>
+        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X10))+SUMPRODUCT(($X$10:$X$14=X10)*($W$10:$W$14&lt;W10))</f>
       </c>
       <c r="Z10" s="5">
         <f>IF(SUMPRODUCT(($X$10:$X$14=X10)*($A$10:$A$14&lt;&gt;A10)*((($W$10:$W$14="")+(W10="")+($W$10:$W$14=W10))&gt;0))&gt;0,1,0)</f>
@@ -3363,7 +3363,7 @@
         <f>J11*10^11+(I11+500)*10^8+U11*10^6+(V11+500)*10^3+G11</f>
       </c>
       <c r="Y11" s="5">
-        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X11))+SUMPRODUCT(($X$10:$X$14=X11)*($W$10:$W$14&lt;&gt;"")*(W11&lt;&gt;"")*($W$10:$W$14&lt;W11))</f>
+        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X11))+SUMPRODUCT(($X$10:$X$14=X11)*($W$10:$W$14&lt;W11))</f>
       </c>
       <c r="Z11" s="5">
         <f>IF(SUMPRODUCT(($X$10:$X$14=X11)*($A$10:$A$14&lt;&gt;A11)*((($W$10:$W$14="")+(W11="")+($W$10:$W$14=W11))&gt;0))&gt;0,1,0)</f>
@@ -3446,7 +3446,7 @@
         <f>J12*10^11+(I12+500)*10^8+U12*10^6+(V12+500)*10^3+G12</f>
       </c>
       <c r="Y12" s="5">
-        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X12))+SUMPRODUCT(($X$10:$X$14=X12)*($W$10:$W$14&lt;&gt;"")*(W12&lt;&gt;"")*($W$10:$W$14&lt;W12))</f>
+        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X12))+SUMPRODUCT(($X$10:$X$14=X12)*($W$10:$W$14&lt;W12))</f>
       </c>
       <c r="Z12" s="5">
         <f>IF(SUMPRODUCT(($X$10:$X$14=X12)*($A$10:$A$14&lt;&gt;A12)*((($W$10:$W$14="")+(W12="")+($W$10:$W$14=W12))&gt;0))&gt;0,1,0)</f>
@@ -3529,7 +3529,7 @@
         <f>J13*10^11+(I13+500)*10^8+U13*10^6+(V13+500)*10^3+G13</f>
       </c>
       <c r="Y13" s="5">
-        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X13))+SUMPRODUCT(($X$10:$X$14=X13)*($W$10:$W$14&lt;&gt;"")*(W13&lt;&gt;"")*($W$10:$W$14&lt;W13))</f>
+        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X13))+SUMPRODUCT(($X$10:$X$14=X13)*($W$10:$W$14&lt;W13))</f>
       </c>
       <c r="Z13" s="5">
         <f>IF(SUMPRODUCT(($X$10:$X$14=X13)*($A$10:$A$14&lt;&gt;A13)*((($W$10:$W$14="")+(W13="")+($W$10:$W$14=W13))&gt;0))&gt;0,1,0)</f>
@@ -3612,7 +3612,7 @@
         <f>J14*10^11+(I14+500)*10^8+U14*10^6+(V14+500)*10^3+G14</f>
       </c>
       <c r="Y14" s="5">
-        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X14))+SUMPRODUCT(($X$10:$X$14=X14)*($W$10:$W$14&lt;&gt;"")*(W14&lt;&gt;"")*($W$10:$W$14&lt;W14))</f>
+        <f>1+SUMPRODUCT(--($X$10:$X$14&gt;X14))+SUMPRODUCT(($X$10:$X$14=X14)*($W$10:$W$14&lt;W14))</f>
       </c>
       <c r="Z14" s="5">
         <f>IF(SUMPRODUCT(($X$10:$X$14=X14)*($A$10:$A$14&lt;&gt;A14)*((($W$10:$W$14="")+(W14="")+($W$10:$W$14=W14))&gt;0))&gt;0,1,0)</f>

</xml_diff>